<commit_message>
260311 commit 重大更新：部署Github Actions
</commit_message>
<xml_diff>
--- a/MSK FETCH/msk_ports.xlsx
+++ b/MSK FETCH/msk_ports.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Files\demo\capaStudy\MSK FETCH\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA5B7B0-72F7-4D9E-A969-C1D24B28D6F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8CCFEB-A863-4E3B-884A-507D80E8800E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5130" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{C7685A01-B79A-4285-B9F8-066FB464F69A}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{C7685A01-B79A-4285-B9F8-066FB464F69A}"/>
   </bookViews>
   <sheets>
     <sheet name="ports" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>city</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -45,144 +45,6 @@
   <si>
     <t>geoid</t>
     <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Shanghai</t>
-  </si>
-  <si>
-    <t>2IW9P6J7XAW72</t>
-  </si>
-  <si>
-    <t>Yantian</t>
-  </si>
-  <si>
-    <t>0L3DBFFJ3KZ9A</t>
-  </si>
-  <si>
-    <t>Tanjung Pelepas</t>
-  </si>
-  <si>
-    <t>2DTLIHUG9YN7S</t>
-  </si>
-  <si>
-    <t>Rotterdam</t>
-  </si>
-  <si>
-    <t>1JUKNJGWHQBNJ</t>
-  </si>
-  <si>
-    <t>Hamburg</t>
-  </si>
-  <si>
-    <t>03KFCBH0IX2TA</t>
-  </si>
-  <si>
-    <t>Antwerp</t>
-  </si>
-  <si>
-    <t>0ZBIURQPE236H</t>
-  </si>
-  <si>
-    <t>London Gateway</t>
-  </si>
-  <si>
-    <t>T4HWDGEKCG3L1</t>
-  </si>
-  <si>
-    <t>Ningbo</t>
-  </si>
-  <si>
-    <t>104T898SJZ6GU</t>
-  </si>
-  <si>
-    <t>Wilhelmshaven</t>
-  </si>
-  <si>
-    <t>1ZPUMHQGZ3KOU</t>
-  </si>
-  <si>
-    <t>Bremerhaven</t>
-  </si>
-  <si>
-    <t>3EX4F5S3MB4OU</t>
-  </si>
-  <si>
-    <t>Algeciras</t>
-  </si>
-  <si>
-    <t>05R47F3DBN69Q</t>
-  </si>
-  <si>
-    <t>Qingdao</t>
-  </si>
-  <si>
-    <t>1YCLYW8V7RZB2</t>
-  </si>
-  <si>
-    <t>Aarhus</t>
-  </si>
-  <si>
-    <t>2RX5LS7KU273Y</t>
-  </si>
-  <si>
-    <t>Gothenburg</t>
-  </si>
-  <si>
-    <t>148LVMHYNW4N3</t>
-  </si>
-  <si>
-    <t>Valencia</t>
-  </si>
-  <si>
-    <t>12LNX9VI6SCYH</t>
-  </si>
-  <si>
-    <t>Barcelona</t>
-  </si>
-  <si>
-    <t>1FQMCYMU9XLZ2</t>
-  </si>
-  <si>
-    <t>La Spezia</t>
-  </si>
-  <si>
-    <t>2743COUCZS8SF</t>
-  </si>
-  <si>
-    <t>Genoa</t>
-  </si>
-  <si>
-    <t>0KSZPEKFXG8ZJ</t>
-  </si>
-  <si>
-    <t>2R3AZ1DW4RJB3</t>
-  </si>
-  <si>
-    <t>Port Said East</t>
-  </si>
-  <si>
-    <t>3I6W2NB2MQV7I</t>
-  </si>
-  <si>
-    <t>Koper</t>
-  </si>
-  <si>
-    <t>2XELE43QKIMIN</t>
-  </si>
-  <si>
-    <t>Rijeka</t>
-  </si>
-  <si>
-    <t>3RIJXP3USK909</t>
-  </si>
-  <si>
-    <t>Gwangyang</t>
-  </si>
-  <si>
-    <t>2XE1KEFDLC8E7</t>
-  </si>
-  <si>
-    <t>Q65JHSTNKPAER</t>
   </si>
   <si>
     <t>AE1</t>
@@ -217,37 +79,207 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Port Tangier</t>
+    <t>Algeciras</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>05R47F3DBN69Q</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Antwerp</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>0ZBIURQPE236H</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Barcelona</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1FQMCYMU9XLZ2</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bremerhaven</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>3EX4F5S3MB4OU</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Busan</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2XOHKM8FX8VI7</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Genoa</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>0KSZPEKFXG8ZJ</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hamburg</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>03KFCBH0IX2TA</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>0FC4MM5Y0O0Z2</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>02W224NQ4IGAE</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jeddah</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>0NJO1NEUBFC7W</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Koper</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2XELE43QKIMIN</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>La Spezia</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2743COUCZS8SF</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>London Gateway</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>T4HWDGEKCG3L1</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ningbo</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>104T898SJZ6GU</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Port Said East</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>3I6W2NB2MQV7I</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Port Tangier Mediterranee</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>0C29F4LWXIITO</t>
-  </si>
-  <si>
-    <t>Vado</t>
-  </si>
-  <si>
-    <t>Port Said</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Qingdao</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1YCLYW8V7RZB2</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rijeka</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>3RIJXP3USK909</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rotterdam</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1JUKNJGWHQBNJ</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shanghai</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2IW9P6J7XAW72</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tanjung Pelepas</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>2DTLIHUG9YN7S</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Valencia</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>12LNX9VI6SCYH</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Wilhelmshaven</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1ZPUMHQGZ3KOU</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <t>Xingang</t>
-  </si>
-  <si>
-    <t>0C7LP1SK8P5TU</t>
-  </si>
-  <si>
-    <t>Busan</t>
-  </si>
-  <si>
-    <t>2XOHKM8FX8VI7</t>
-  </si>
-  <si>
-    <t>Port Tangier Mediterranee</t>
-  </si>
-  <si>
-    <t>Jeddah</t>
-  </si>
-  <si>
-    <t>0NJO1NEUBFC7W</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Yantian</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>0L3DBFFJ3KZ9A</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>02GYFH4R8RVY6</t>
+  </si>
+  <si>
+    <t>Genoa Vado Ligure</t>
+  </si>
+  <si>
+    <t>19UUBIUIHO0TG</t>
+  </si>
+  <si>
+    <t>Ambarli Port Istanbul</t>
+  </si>
+  <si>
+    <t>Izmit Korfezi</t>
   </si>
 </sst>
 </file>
@@ -649,8 +681,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7413BB00-6B5B-4ED0-87FD-3EA41C705E43}">
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="26.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.73046875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.5">
       <c r="A1" s="1" t="s">
@@ -660,252 +696,236 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.5">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.5">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15" x14ac:dyDescent="0.5">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.5">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="15" x14ac:dyDescent="0.5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="15" x14ac:dyDescent="0.5">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A10" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A16" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A18" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A19" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A23" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A25" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A26" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" s="1" customFormat="1" ht="15" x14ac:dyDescent="0.5">
+      <c r="A27" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A13" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A14" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A15" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A16" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A17" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A18" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A19" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A20" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A21" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A22" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A23" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A24" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A25" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A26" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A27" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="28" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A28" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>57</v>
-      </c>
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
     </row>
     <row r="29" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A29" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>40</v>
-      </c>
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
     </row>
     <row r="30" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A30" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>66</v>
-      </c>
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
     </row>
     <row r="31" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A31" s="1"/>
+      <c r="A31" s="2"/>
       <c r="B31" s="1"/>
     </row>
     <row r="32" spans="1:2" ht="15" x14ac:dyDescent="0.5">
       <c r="A32" s="2"/>
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="1:2" ht="15" x14ac:dyDescent="0.5">
-      <c r="A33" s="2"/>
-      <c r="B33" s="1"/>
-    </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -917,42 +937,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>